<commit_message>
updated okn 17th April 2026
</commit_message>
<xml_diff>
--- a/Programming and Concepts/DSA 450/FINAL450.xlsx
+++ b/Programming and Concepts/DSA 450/FINAL450.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Documents\Programming\CP GIT\Competitive-Programming\Programming and Concepts\DSA 450\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{679C74F2-E6AA-437F-B2FF-EE4D981D5B2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90BEF363-897E-4A97-88B5-85151B61C78B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1362" uniqueCount="487">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1367" uniqueCount="492">
   <si>
     <t>Questions by Love Babbar:</t>
   </si>
@@ -1481,6 +1481,21 @@
   </si>
   <si>
     <t xml:space="preserve">Transposed matrix  optimal solution remaining </t>
+  </si>
+  <si>
+    <t xml:space="preserve">didn’t solve the alternative solution </t>
+  </si>
+  <si>
+    <t>need some revision and practice again (had to see the optimised code with logic)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">use of 2 stacks here for iterative postorder traversal </t>
+  </si>
+  <si>
+    <t xml:space="preserve">print only the right element of the respective level in the level order traversal </t>
+  </si>
+  <si>
+    <t xml:space="preserve">print only the left element of the respective level in the level order traversal </t>
   </si>
 </sst>
 </file>
@@ -3855,179 +3870,188 @@
       <c r="B176" s="18"/>
       <c r="C176" s="12"/>
     </row>
-    <row r="177" spans="1:3">
+    <row r="177" spans="1:4">
       <c r="A177" s="8" t="s">
         <v>189</v>
       </c>
       <c r="B177" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="C177" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="178" spans="1:3">
+      <c r="C177" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4">
       <c r="A178" s="8" t="s">
         <v>189</v>
       </c>
       <c r="B178" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="C178" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="179" spans="1:3">
+      <c r="C178" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4">
       <c r="A179" s="8" t="s">
         <v>189</v>
       </c>
       <c r="B179" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="C179" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="180" spans="1:3">
+      <c r="C179" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4">
       <c r="A180" s="8" t="s">
         <v>189</v>
       </c>
       <c r="B180" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="C180" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="181" spans="1:3">
+      <c r="C180" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="181" spans="1:4">
       <c r="A181" s="8" t="s">
         <v>189</v>
       </c>
       <c r="B181" s="9" t="s">
         <v>194</v>
       </c>
-      <c r="C181" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="182" spans="1:3">
+      <c r="C181" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4">
       <c r="A182" s="8" t="s">
         <v>189</v>
       </c>
       <c r="B182" s="9" t="s">
         <v>195</v>
       </c>
-      <c r="C182" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="183" spans="1:3">
+      <c r="C182" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4">
       <c r="A183" s="8" t="s">
         <v>189</v>
       </c>
       <c r="B183" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="C183" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="184" spans="1:3">
+      <c r="C183" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="184" spans="1:4">
       <c r="A184" s="8" t="s">
         <v>189</v>
       </c>
       <c r="B184" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="C184" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="185" spans="1:3">
+      <c r="C184" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D184" s="1" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="185" spans="1:4">
       <c r="A185" s="8" t="s">
         <v>189</v>
       </c>
       <c r="B185" s="9" t="s">
         <v>198</v>
       </c>
-      <c r="C185" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="186" spans="1:3">
+      <c r="C185" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D185" s="1" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4">
       <c r="A186" s="8" t="s">
         <v>189</v>
       </c>
       <c r="B186" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="C186" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="187" spans="1:3">
+      <c r="C186" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D186" s="1" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4">
       <c r="A187" s="8" t="s">
         <v>189</v>
       </c>
       <c r="B187" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="C187" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="188" spans="1:3">
+      <c r="C187" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="188" spans="1:4">
       <c r="A188" s="8" t="s">
         <v>189</v>
       </c>
       <c r="B188" s="9" t="s">
         <v>201</v>
       </c>
-      <c r="C188" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="189" spans="1:3">
+      <c r="C188" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4">
       <c r="A189" s="8" t="s">
         <v>189</v>
       </c>
       <c r="B189" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="C189" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="190" spans="1:3">
+      <c r="C189" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="190" spans="1:4">
       <c r="A190" s="8" t="s">
         <v>189</v>
       </c>
       <c r="B190" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="C190" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="191" spans="1:3">
+      <c r="C190" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="191" spans="1:4">
       <c r="A191" s="8" t="s">
         <v>189</v>
       </c>
       <c r="B191" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="C191" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="192" spans="1:3">
+      <c r="C191" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="192" spans="1:4">
       <c r="A192" s="8" t="s">
         <v>189</v>
       </c>
       <c r="B192" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="C192" s="12" t="s">
+      <c r="C192" s="10" t="s">
         <v>17</v>
       </c>
     </row>
@@ -5047,7 +5071,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="289" spans="1:3">
+    <row r="289" spans="1:4">
       <c r="A289" s="8" t="s">
         <v>283</v>
       </c>
@@ -5058,7 +5082,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="290" spans="1:3">
+    <row r="290" spans="1:4">
       <c r="A290" s="8" t="s">
         <v>283</v>
       </c>
@@ -5069,7 +5093,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="291" spans="1:3">
+    <row r="291" spans="1:4">
       <c r="A291" s="8" t="s">
         <v>283</v>
       </c>
@@ -5080,7 +5104,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="292" spans="1:3">
+    <row r="292" spans="1:4">
       <c r="A292" s="8" t="s">
         <v>283</v>
       </c>
@@ -5091,7 +5115,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="293" spans="1:3">
+    <row r="293" spans="1:4">
       <c r="A293" s="8" t="s">
         <v>283</v>
       </c>
@@ -5102,59 +5126,62 @@
         <v>17</v>
       </c>
     </row>
-    <row r="294" spans="1:3">
+    <row r="294" spans="1:4">
       <c r="B294" s="18"/>
       <c r="C294" s="12"/>
     </row>
-    <row r="295" spans="1:3">
+    <row r="295" spans="1:4">
       <c r="B295" s="18"/>
       <c r="C295" s="12"/>
     </row>
-    <row r="296" spans="1:3">
+    <row r="296" spans="1:4">
       <c r="A296" s="8" t="s">
         <v>303</v>
       </c>
       <c r="B296" s="9" t="s">
         <v>304</v>
       </c>
-      <c r="C296" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="297" spans="1:3">
+      <c r="C296" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="297" spans="1:4">
       <c r="A297" s="8" t="s">
         <v>303</v>
       </c>
       <c r="B297" s="9" t="s">
         <v>305</v>
       </c>
-      <c r="C297" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="298" spans="1:3">
+      <c r="C297" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="298" spans="1:4">
       <c r="A298" s="8" t="s">
         <v>303</v>
       </c>
       <c r="B298" s="9" t="s">
         <v>306</v>
       </c>
-      <c r="C298" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="299" spans="1:3">
+      <c r="C298" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="299" spans="1:4">
       <c r="A299" s="8" t="s">
         <v>303</v>
       </c>
       <c r="B299" s="9" t="s">
         <v>307</v>
       </c>
-      <c r="C299" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="300" spans="1:3">
+      <c r="C299" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D299" s="1" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="300" spans="1:4">
       <c r="A300" s="8" t="s">
         <v>303</v>
       </c>
@@ -5165,40 +5192,43 @@
         <v>17</v>
       </c>
     </row>
-    <row r="301" spans="1:3">
+    <row r="301" spans="1:4">
       <c r="A301" s="8" t="s">
         <v>303</v>
       </c>
       <c r="B301" s="9" t="s">
         <v>309</v>
       </c>
-      <c r="C301" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="302" spans="1:3">
+      <c r="C301" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="302" spans="1:4">
       <c r="A302" s="8" t="s">
         <v>303</v>
       </c>
       <c r="B302" s="9" t="s">
         <v>310</v>
       </c>
-      <c r="C302" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="303" spans="1:3">
+      <c r="C302" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="303" spans="1:4">
       <c r="A303" s="8" t="s">
         <v>303</v>
       </c>
       <c r="B303" s="9" t="s">
         <v>311</v>
       </c>
-      <c r="C303" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="304" spans="1:3">
+      <c r="C303" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D303" s="1" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="304" spans="1:4">
       <c r="A304" s="8" t="s">
         <v>303</v>
       </c>

</xml_diff>

<commit_message>
Update 24th August 2026
</commit_message>
<xml_diff>
--- a/Programming and Concepts/DSA 450/FINAL450.xlsx
+++ b/Programming and Concepts/DSA 450/FINAL450.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Documents\Programming\CP GIT\Competitive-Programming\Programming and Concepts\DSA 450\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\STORAGE\Work\DSA\Competitive-Programming\Programming and Concepts\DSA 450\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90BEF363-897E-4A97-88B5-85151B61C78B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A947A7C-C358-4E95-B956-63057E698DF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3499,7 +3499,7 @@
       <c r="B141" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="C141" s="12" t="s">
+      <c r="C141" s="10" t="s">
         <v>17</v>
       </c>
     </row>
@@ -3532,7 +3532,7 @@
       <c r="B144" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="C144" s="12" t="s">
+      <c r="C144" s="10" t="s">
         <v>17</v>
       </c>
     </row>
@@ -3543,7 +3543,7 @@
       <c r="B145" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="C145" s="12" t="s">
+      <c r="C145" s="10" t="s">
         <v>17</v>
       </c>
     </row>
@@ -3554,7 +3554,7 @@
       <c r="B146" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="C146" s="12" t="s">
+      <c r="C146" s="10" t="s">
         <v>17</v>
       </c>
     </row>
@@ -3565,7 +3565,7 @@
       <c r="B147" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="C147" s="12" t="s">
+      <c r="C147" s="10" t="s">
         <v>17</v>
       </c>
     </row>
@@ -3576,7 +3576,7 @@
       <c r="B148" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="C148" s="12" t="s">
+      <c r="C148" s="10" t="s">
         <v>17</v>
       </c>
     </row>
@@ -3587,7 +3587,7 @@
       <c r="B149" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="C149" s="12" t="s">
+      <c r="C149" s="10" t="s">
         <v>17</v>
       </c>
     </row>
@@ -3598,7 +3598,7 @@
       <c r="B150" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="C150" s="12" t="s">
+      <c r="C150" s="10" t="s">
         <v>17</v>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       <c r="B153" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="C153" s="12" t="s">
+      <c r="C153" s="10" t="s">
         <v>17</v>
       </c>
     </row>
@@ -3642,7 +3642,7 @@
       <c r="B154" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="C154" s="12" t="s">
+      <c r="C154" s="10" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 24th September 2026, linked list
</commit_message>
<xml_diff>
--- a/Programming and Concepts/DSA 450/FINAL450.xlsx
+++ b/Programming and Concepts/DSA 450/FINAL450.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\STORAGE\Work\DSA\Competitive-Programming\Programming and Concepts\DSA 450\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A947A7C-C358-4E95-B956-63057E698DF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAC52304-14A0-4EDE-878E-36E45BF1A949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3510,7 +3510,7 @@
       <c r="B142" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="C142" s="12" t="s">
+      <c r="C142" s="10" t="s">
         <v>17</v>
       </c>
     </row>
@@ -3521,7 +3521,7 @@
       <c r="B143" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="C143" s="12" t="s">
+      <c r="C143" s="10" t="s">
         <v>17</v>
       </c>
     </row>
@@ -3653,7 +3653,7 @@
       <c r="B155" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="C155" s="12" t="s">
+      <c r="C155" s="10" t="s">
         <v>17</v>
       </c>
     </row>
@@ -3664,7 +3664,7 @@
       <c r="B156" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="C156" s="12" t="s">
+      <c r="C156" s="10" t="s">
         <v>17</v>
       </c>
     </row>
@@ -3675,7 +3675,7 @@
       <c r="B157" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="C157" s="12" t="s">
+      <c r="C157" s="10" t="s">
         <v>17</v>
       </c>
     </row>
@@ -3785,7 +3785,7 @@
       <c r="B167" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="C167" s="12" t="s">
+      <c r="C167" s="10" t="s">
         <v>17</v>
       </c>
     </row>
@@ -3840,7 +3840,7 @@
       <c r="B172" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="C172" s="12" t="s">
+      <c r="C172" s="10" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>